<commit_message>
Add 9 new artworks to gallery
Adds Strange Loop, Seascape, Control Panel, Laundry, Can Abstraction,
Happy Bday, Seascape Triptych, untitled2, and Summer Groceries — including
all corresponding thumbnail and detail images.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Artwork_info.xlsx
+++ b/Artwork_info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joeyj\OneDrive\Documents\Claude_Code\website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B346D1CC-C728-4D28-88D1-634D0B3DD58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F20BE8-05A2-4B0E-BAE0-3065AC06DFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{45523018-7D47-4FC1-99C3-F79E30ED753A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="91">
   <si>
     <t>Artwork_Name</t>
   </si>
@@ -256,6 +256,57 @@
   </si>
   <si>
     <t>A standing man reading a red light mask</t>
+  </si>
+  <si>
+    <t>Untitled 2</t>
+  </si>
+  <si>
+    <t>A secction of a tennis court in blue/green</t>
+  </si>
+  <si>
+    <t>Strange Loop</t>
+  </si>
+  <si>
+    <t>Three old fashioneds, three orange slices, and a burning candle</t>
+  </si>
+  <si>
+    <t>Seascape</t>
+  </si>
+  <si>
+    <t>An abstract landscape in various shades of blue</t>
+  </si>
+  <si>
+    <t>Control Panel</t>
+  </si>
+  <si>
+    <t>A grey control panel standing in front of the ocean</t>
+  </si>
+  <si>
+    <t>Laundry</t>
+  </si>
+  <si>
+    <t>4 x 4</t>
+  </si>
+  <si>
+    <t>Can Abstraction</t>
+  </si>
+  <si>
+    <t>A stretched out can with a red background</t>
+  </si>
+  <si>
+    <t>Folded laundry with a yellow background</t>
+  </si>
+  <si>
+    <t>Happy Bday</t>
+  </si>
+  <si>
+    <t>A birthday cake with lit candles on top, with a dark background</t>
+  </si>
+  <si>
+    <t>Seascape Triptych</t>
+  </si>
+  <si>
+    <t>Three small ocean landscape paintings</t>
   </si>
 </sst>
 </file>
@@ -625,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EABF6B0-7F9A-49C9-BF10-DB049849EF3C}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -1093,6 +1144,142 @@
         <v>73</v>
       </c>
     </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28">
+        <v>2015</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>2026</v>
+      </c>
+      <c r="E29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30">
+        <v>2024</v>
+      </c>
+      <c r="E30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31">
+        <v>2024</v>
+      </c>
+      <c r="E31" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32">
+        <v>2024</v>
+      </c>
+      <c r="E32" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33">
+        <v>2024</v>
+      </c>
+      <c r="E33" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34">
+        <v>2024</v>
+      </c>
+      <c r="E34" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B35" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35">
+        <v>2021</v>
+      </c>
+      <c r="E35" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Commit miscellaneous project files
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Artwork_info.xlsx
+++ b/Artwork_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joeyj\OneDrive\Documents\Claude_Code\website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F20BE8-05A2-4B0E-BAE0-3065AC06DFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC7B212-252E-4B31-B7C2-1DCDF377C822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{45523018-7D47-4FC1-99C3-F79E30ED753A}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t>Ocean waves crashing on a beach, with a dark sky in the background</t>
   </si>
   <si>
-    <t>What's in the Cabinet</t>
-  </si>
-  <si>
     <t>16 x 20</t>
   </si>
   <si>
@@ -307,6 +304,9 @@
   </si>
   <si>
     <t>Three small ocean landscape paintings</t>
+  </si>
+  <si>
+    <t>Cabinet</t>
   </si>
 </sst>
 </file>
@@ -806,10 +806,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" t="s">
         <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -818,12 +818,12 @@
         <v>2024</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
@@ -835,15 +835,15 @@
         <v>2024</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
         <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -852,15 +852,15 @@
         <v>2024</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
       </c>
       <c r="C11" t="s">
         <v>7</v>
@@ -869,15 +869,15 @@
         <v>2024</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
@@ -886,15 +886,15 @@
         <v>2024</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" t="s">
-        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>7</v>
@@ -903,12 +903,12 @@
         <v>2023</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>
@@ -920,12 +920,12 @@
         <v>2023</v>
       </c>
       <c r="E14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
@@ -937,12 +937,12 @@
         <v>2022</v>
       </c>
       <c r="E15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
@@ -954,32 +954,32 @@
         <v>2022</v>
       </c>
       <c r="E16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>48</v>
-      </c>
-      <c r="C17" t="s">
-        <v>49</v>
       </c>
       <c r="D17">
         <v>2022</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" t="s">
         <v>51</v>
-      </c>
-      <c r="B18" t="s">
-        <v>52</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
@@ -988,15 +988,15 @@
         <v>2023</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" t="s">
         <v>54</v>
-      </c>
-      <c r="B19" t="s">
-        <v>55</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
@@ -1005,131 +1005,131 @@
         <v>2022</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D20">
         <v>2018</v>
       </c>
       <c r="E20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21">
         <v>2017</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" t="s">
         <v>61</v>
       </c>
-      <c r="B22" t="s">
-        <v>62</v>
-      </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D22">
         <v>2015</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s">
         <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D23">
         <v>2021</v>
       </c>
       <c r="E23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
         <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D24">
         <v>2021</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" t="s">
         <v>19</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25">
         <v>2021</v>
       </c>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D26">
         <v>2021</v>
       </c>
       <c r="E26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
         <v>19</v>
@@ -1141,29 +1141,29 @@
         <v>2026</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D28">
         <v>2015</v>
       </c>
       <c r="E28" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
         <v>16</v>
@@ -1175,49 +1175,49 @@
         <v>2026</v>
       </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D30">
         <v>2024</v>
       </c>
       <c r="E30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D31">
         <v>2024</v>
       </c>
       <c r="E31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" t="s">
         <v>82</v>
-      </c>
-      <c r="B32" t="s">
-        <v>83</v>
       </c>
       <c r="C32" t="s">
         <v>20</v>
@@ -1226,15 +1226,15 @@
         <v>2024</v>
       </c>
       <c r="E32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B33" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C33" t="s">
         <v>20</v>
@@ -1243,41 +1243,41 @@
         <v>2024</v>
       </c>
       <c r="E33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B34" t="s">
         <v>19</v>
       </c>
       <c r="C34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D34">
         <v>2024</v>
       </c>
       <c r="E34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D35">
         <v>2021</v>
       </c>
       <c r="E35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>